<commit_message>
Update MLB hitter fantasy scores 2026-07-12 (2026-07-14 01:50 AM)
</commit_message>
<xml_diff>
--- a/PRIZEPICKS_HITTER_AI_V4_TOP30_2026_07_12.xlsx
+++ b/PRIZEPICKS_HITTER_AI_V4_TOP30_2026_07_12.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hitter Model" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hitter Model'!$A$1:$GB$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hitter Model'!$A$1:$HC$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:GB31"/>
+  <dimension ref="A1:HC31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -697,6 +697,33 @@
     <col width="13" customWidth="1" min="182" max="182"/>
     <col width="13" customWidth="1" min="183" max="183"/>
     <col width="12" customWidth="1" min="184" max="184"/>
+    <col width="12" customWidth="1" min="185" max="185"/>
+    <col width="12" customWidth="1" min="186" max="186"/>
+    <col width="12" customWidth="1" min="187" max="187"/>
+    <col width="12" customWidth="1" min="188" max="188"/>
+    <col width="12" customWidth="1" min="189" max="189"/>
+    <col width="12" customWidth="1" min="190" max="190"/>
+    <col width="12" customWidth="1" min="191" max="191"/>
+    <col width="12" customWidth="1" min="192" max="192"/>
+    <col width="12" customWidth="1" min="193" max="193"/>
+    <col width="12" customWidth="1" min="194" max="194"/>
+    <col width="12" customWidth="1" min="195" max="195"/>
+    <col width="12" customWidth="1" min="196" max="196"/>
+    <col width="12" customWidth="1" min="197" max="197"/>
+    <col width="12" customWidth="1" min="198" max="198"/>
+    <col width="12" customWidth="1" min="199" max="199"/>
+    <col width="12" customWidth="1" min="200" max="200"/>
+    <col width="12" customWidth="1" min="201" max="201"/>
+    <col width="12" customWidth="1" min="202" max="202"/>
+    <col width="12" customWidth="1" min="203" max="203"/>
+    <col width="12" customWidth="1" min="204" max="204"/>
+    <col width="12" customWidth="1" min="205" max="205"/>
+    <col width="12" customWidth="1" min="206" max="206"/>
+    <col width="12" customWidth="1" min="207" max="207"/>
+    <col width="12" customWidth="1" min="208" max="208"/>
+    <col width="12" customWidth="1" min="209" max="209"/>
+    <col width="12" customWidth="1" min="210" max="210"/>
+    <col width="12" customWidth="1" min="211" max="211"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1617,6 +1644,141 @@
       </c>
       <c r="GB1" s="2" t="inlineStr">
         <is>
+          <t>Floor Uplift 2.5 FS</t>
+        </is>
+      </c>
+      <c r="GC1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 3.0 FS</t>
+        </is>
+      </c>
+      <c r="GD1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 3.5 FS</t>
+        </is>
+      </c>
+      <c r="GE1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 4.0 FS</t>
+        </is>
+      </c>
+      <c r="GF1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 4.5 FS</t>
+        </is>
+      </c>
+      <c r="GG1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 5.0 FS</t>
+        </is>
+      </c>
+      <c r="GH1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 5.5 FS</t>
+        </is>
+      </c>
+      <c r="GI1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 6.0 FS</t>
+        </is>
+      </c>
+      <c r="GJ1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 6.5 FS</t>
+        </is>
+      </c>
+      <c r="GK1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 7.0 FS</t>
+        </is>
+      </c>
+      <c r="GL1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 7.5 FS</t>
+        </is>
+      </c>
+      <c r="GM1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 8.0 FS</t>
+        </is>
+      </c>
+      <c r="GN1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 8.5 FS</t>
+        </is>
+      </c>
+      <c r="GO1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 9.0 FS</t>
+        </is>
+      </c>
+      <c r="GP1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 9.5 FS</t>
+        </is>
+      </c>
+      <c r="GQ1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 10.0 FS</t>
+        </is>
+      </c>
+      <c r="GR1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 10.5 FS</t>
+        </is>
+      </c>
+      <c r="GS1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 11.0 FS</t>
+        </is>
+      </c>
+      <c r="GT1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 11.5 FS</t>
+        </is>
+      </c>
+      <c r="GU1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 12.0 FS</t>
+        </is>
+      </c>
+      <c r="GV1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 12.5 FS</t>
+        </is>
+      </c>
+      <c r="GW1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 13.0 FS</t>
+        </is>
+      </c>
+      <c r="GX1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 13.5 FS</t>
+        </is>
+      </c>
+      <c r="GY1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 14.0 FS</t>
+        </is>
+      </c>
+      <c r="GZ1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 14.5 FS</t>
+        </is>
+      </c>
+      <c r="HA1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 15.0 FS</t>
+        </is>
+      </c>
+      <c r="HB1" s="2" t="inlineStr">
+        <is>
+          <t>Floor Uplift 15.5 FS</t>
+        </is>
+      </c>
+      <c r="HC1" s="2" t="inlineStr">
+        <is>
           <t>Confidence</t>
         </is>
       </c>
@@ -1694,40 +1856,40 @@
         </is>
       </c>
       <c r="R2" s="5" t="n">
-        <v>85.3</v>
+        <v>91.2</v>
       </c>
       <c r="S2" s="5" t="n">
-        <v>79.7</v>
+        <v>87.7</v>
       </c>
       <c r="T2" s="5" t="n">
-        <v>79.7</v>
+        <v>87.2</v>
       </c>
       <c r="U2" s="5" t="n">
-        <v>74.40000000000001</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="V2" s="5" t="n">
-        <v>74.40000000000001</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="W2" s="5" t="n">
-        <v>67.09999999999999</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="X2" s="5" t="n">
-        <v>67.09999999999999</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="Y2" s="5" t="n">
-        <v>63.5</v>
+        <v>67.5</v>
       </c>
       <c r="Z2" s="5" t="n">
-        <v>63.5</v>
-      </c>
-      <c r="AA2" s="6" t="n">
-        <v>56</v>
-      </c>
-      <c r="AB2" s="7" t="n">
-        <v>56</v>
-      </c>
-      <c r="AC2" s="7" t="n">
-        <v>52</v>
+        <v>67</v>
+      </c>
+      <c r="AA2" s="5" t="n">
+        <v>59</v>
+      </c>
+      <c r="AB2" s="5" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="AC2" s="6" t="n">
+        <v>53</v>
       </c>
       <c r="AD2" s="7" t="n">
         <v>52</v>
@@ -1775,7 +1937,7 @@
         <v>29.4</v>
       </c>
       <c r="AS2" s="3" t="n">
-        <v>299.26</v>
+        <v>299.98</v>
       </c>
       <c r="AT2" s="4" t="inlineStr">
         <is>
@@ -2221,7 +2383,88 @@
       <c r="GA2" s="3" t="n">
         <v>29.4</v>
       </c>
-      <c r="GB2" s="4" t="inlineStr">
+      <c r="GB2" s="3" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="GC2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD2" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE2" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF2" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG2" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH2" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ2" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK2" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL2" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC2" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2300,40 +2543,40 @@
         </is>
       </c>
       <c r="R3" s="5" t="n">
-        <v>85.59999999999999</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="S3" s="5" t="n">
-        <v>80.40000000000001</v>
+        <v>88.2</v>
       </c>
       <c r="T3" s="5" t="n">
-        <v>80.40000000000001</v>
+        <v>87.8</v>
       </c>
       <c r="U3" s="5" t="n">
-        <v>75.09999999999999</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="V3" s="5" t="n">
-        <v>75.09999999999999</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="W3" s="5" t="n">
-        <v>67.59999999999999</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="X3" s="5" t="n">
-        <v>67.59999999999999</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="Y3" s="5" t="n">
-        <v>63.5</v>
+        <v>67.5</v>
       </c>
       <c r="Z3" s="5" t="n">
-        <v>63.5</v>
-      </c>
-      <c r="AA3" s="6" t="n">
-        <v>56.3</v>
-      </c>
-      <c r="AB3" s="7" t="n">
-        <v>56.3</v>
-      </c>
-      <c r="AC3" s="7" t="n">
-        <v>51.9</v>
+        <v>67</v>
+      </c>
+      <c r="AA3" s="5" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="AB3" s="5" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="AC3" s="6" t="n">
+        <v>52.9</v>
       </c>
       <c r="AD3" s="7" t="n">
         <v>51.9</v>
@@ -2381,7 +2624,7 @@
         <v>27.4</v>
       </c>
       <c r="AS3" s="3" t="n">
-        <v>283.86</v>
+        <v>284.58</v>
       </c>
       <c r="AT3" s="4" t="inlineStr">
         <is>
@@ -2827,7 +3070,88 @@
       <c r="GA3" s="3" t="n">
         <v>27.4</v>
       </c>
-      <c r="GB3" s="4" t="inlineStr">
+      <c r="GB3" s="3" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="GC3" s="3" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="GD3" s="3" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="GE3" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF3" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG3" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH3" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI3" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ3" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK3" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL3" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC3" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2906,40 +3230,40 @@
         </is>
       </c>
       <c r="R4" s="5" t="n">
-        <v>84.40000000000001</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="S4" s="5" t="n">
-        <v>77.7</v>
+        <v>85.7</v>
       </c>
       <c r="T4" s="5" t="n">
-        <v>77.7</v>
+        <v>85.2</v>
       </c>
       <c r="U4" s="5" t="n">
-        <v>73.40000000000001</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="V4" s="5" t="n">
-        <v>73.40000000000001</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="W4" s="5" t="n">
-        <v>64.90000000000001</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="X4" s="5" t="n">
-        <v>64.90000000000001</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="Y4" s="5" t="n">
-        <v>61.5</v>
+        <v>65.5</v>
       </c>
       <c r="Z4" s="5" t="n">
-        <v>61.5</v>
+        <v>65</v>
       </c>
       <c r="AA4" s="6" t="n">
-        <v>54.5</v>
+        <v>57.5</v>
       </c>
       <c r="AB4" s="7" t="n">
-        <v>54.5</v>
+        <v>57</v>
       </c>
       <c r="AC4" s="7" t="n">
-        <v>49.7</v>
+        <v>50.7</v>
       </c>
       <c r="AD4" s="7" t="n">
         <v>49.7</v>
@@ -2987,7 +3311,7 @@
         <v>25.7</v>
       </c>
       <c r="AS4" s="3" t="n">
-        <v>279.93</v>
+        <v>280.65</v>
       </c>
       <c r="AT4" s="4" t="inlineStr">
         <is>
@@ -3427,7 +3751,88 @@
       <c r="GA4" s="3" t="n">
         <v>25.7</v>
       </c>
-      <c r="GB4" s="4" t="inlineStr">
+      <c r="GB4" s="3" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="GC4" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD4" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE4" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF4" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH4" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI4" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ4" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL4" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC4" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3506,40 +3911,40 @@
         </is>
       </c>
       <c r="R5" s="5" t="n">
-        <v>82.5</v>
+        <v>89.5</v>
       </c>
       <c r="S5" s="5" t="n">
-        <v>76.2</v>
+        <v>84.2</v>
       </c>
       <c r="T5" s="5" t="n">
-        <v>76.2</v>
+        <v>83.7</v>
       </c>
       <c r="U5" s="5" t="n">
-        <v>71.40000000000001</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="V5" s="5" t="n">
-        <v>71.40000000000001</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="W5" s="5" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="X5" s="5" t="n">
-        <v>63</v>
+        <v>67.5</v>
       </c>
       <c r="Y5" s="5" t="n">
-        <v>59.3</v>
+        <v>63.3</v>
       </c>
       <c r="Z5" s="5" t="n">
-        <v>59.3</v>
+        <v>62.8</v>
       </c>
       <c r="AA5" s="6" t="n">
-        <v>52.6</v>
+        <v>55.6</v>
       </c>
       <c r="AB5" s="7" t="n">
-        <v>52.6</v>
+        <v>55.1</v>
       </c>
       <c r="AC5" s="7" t="n">
-        <v>48.8</v>
+        <v>49.8</v>
       </c>
       <c r="AD5" s="7" t="n">
         <v>48.8</v>
@@ -3587,7 +3992,7 @@
         <v>29</v>
       </c>
       <c r="AS5" s="3" t="n">
-        <v>272.38</v>
+        <v>273.1</v>
       </c>
       <c r="AT5" s="4" t="inlineStr">
         <is>
@@ -4027,7 +4432,88 @@
       <c r="GA5" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="GB5" s="4" t="inlineStr">
+      <c r="GB5" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GC5" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD5" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE5" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF5" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH5" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ5" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL5" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC5" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -4106,40 +4592,40 @@
         </is>
       </c>
       <c r="R6" s="5" t="n">
-        <v>74.5</v>
+        <v>82.5</v>
       </c>
       <c r="S6" s="5" t="n">
-        <v>65.40000000000001</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="T6" s="5" t="n">
-        <v>65.40000000000001</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="U6" s="5" t="n">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="V6" s="5" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="W6" s="6" t="n">
-        <v>52.4</v>
+        <v>57.4</v>
       </c>
       <c r="X6" s="7" t="n">
-        <v>52.4</v>
+        <v>56.9</v>
       </c>
       <c r="Y6" s="7" t="n">
-        <v>49.8</v>
+        <v>53.8</v>
       </c>
       <c r="Z6" s="7" t="n">
-        <v>49.8</v>
+        <v>53.3</v>
       </c>
       <c r="AA6" s="7" t="n">
-        <v>43.1</v>
+        <v>46.1</v>
       </c>
       <c r="AB6" s="7" t="n">
-        <v>43.1</v>
+        <v>45.6</v>
       </c>
       <c r="AC6" s="7" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="AD6" s="7" t="n">
         <v>40</v>
@@ -4187,7 +4673,7 @@
         <v>23.2</v>
       </c>
       <c r="AS6" s="3" t="n">
-        <v>263.52</v>
+        <v>264.24</v>
       </c>
       <c r="AT6" s="4" t="inlineStr">
         <is>
@@ -4633,7 +5119,88 @@
       <c r="GA6" s="3" t="n">
         <v>23.2</v>
       </c>
-      <c r="GB6" s="4" t="inlineStr">
+      <c r="GB6" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC6" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD6" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE6" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF6" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH6" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ6" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK6" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL6" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC6" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -4712,40 +5279,40 @@
         </is>
       </c>
       <c r="R7" s="5" t="n">
-        <v>86.2</v>
+        <v>91.7</v>
       </c>
       <c r="S7" s="5" t="n">
-        <v>78.3</v>
+        <v>86.3</v>
       </c>
       <c r="T7" s="5" t="n">
-        <v>78.3</v>
+        <v>85.8</v>
       </c>
       <c r="U7" s="5" t="n">
-        <v>75.90000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="V7" s="5" t="n">
-        <v>75.90000000000001</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="W7" s="5" t="n">
-        <v>65.90000000000001</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="X7" s="5" t="n">
-        <v>65.90000000000001</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="Y7" s="5" t="n">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="Z7" s="5" t="n">
-        <v>63</v>
-      </c>
-      <c r="AA7" s="6" t="n">
-        <v>56.3</v>
-      </c>
-      <c r="AB7" s="7" t="n">
-        <v>56.3</v>
-      </c>
-      <c r="AC7" s="7" t="n">
-        <v>50.2</v>
+        <v>66.5</v>
+      </c>
+      <c r="AA7" s="5" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="AB7" s="5" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="AC7" s="6" t="n">
+        <v>51.2</v>
       </c>
       <c r="AD7" s="7" t="n">
         <v>50.2</v>
@@ -4793,7 +5360,7 @@
         <v>24.9</v>
       </c>
       <c r="AS7" s="3" t="n">
-        <v>263.19</v>
+        <v>263.91</v>
       </c>
       <c r="AT7" s="4" t="inlineStr">
         <is>
@@ -5239,7 +5806,88 @@
       <c r="GA7" s="3" t="n">
         <v>24.9</v>
       </c>
-      <c r="GB7" s="4" t="inlineStr">
+      <c r="GB7" s="3" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="GC7" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD7" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH7" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI7" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ7" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL7" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC7" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -5318,40 +5966,40 @@
         </is>
       </c>
       <c r="R8" s="5" t="n">
-        <v>83.2</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="S8" s="5" t="n">
-        <v>75.8</v>
+        <v>83.8</v>
       </c>
       <c r="T8" s="5" t="n">
-        <v>75.8</v>
+        <v>83.3</v>
       </c>
       <c r="U8" s="5" t="n">
-        <v>71.7</v>
+        <v>78.7</v>
       </c>
       <c r="V8" s="5" t="n">
-        <v>71.7</v>
+        <v>77.7</v>
       </c>
       <c r="W8" s="5" t="n">
-        <v>62.8</v>
+        <v>67.8</v>
       </c>
       <c r="X8" s="5" t="n">
-        <v>62.8</v>
+        <v>67.3</v>
       </c>
       <c r="Y8" s="5" t="n">
-        <v>59.4</v>
+        <v>63.4</v>
       </c>
       <c r="Z8" s="5" t="n">
-        <v>59.4</v>
+        <v>62.9</v>
       </c>
       <c r="AA8" s="6" t="n">
-        <v>52.1</v>
+        <v>55.1</v>
       </c>
       <c r="AB8" s="7" t="n">
-        <v>52.1</v>
+        <v>54.6</v>
       </c>
       <c r="AC8" s="7" t="n">
-        <v>47.5</v>
+        <v>48.5</v>
       </c>
       <c r="AD8" s="7" t="n">
         <v>47.5</v>
@@ -5399,7 +6047,7 @@
         <v>24.7</v>
       </c>
       <c r="AS8" s="3" t="n">
-        <v>262.31</v>
+        <v>263.03</v>
       </c>
       <c r="AT8" s="4" t="inlineStr">
         <is>
@@ -5845,7 +6493,88 @@
       <c r="GA8" s="3" t="n">
         <v>24.7</v>
       </c>
-      <c r="GB8" s="4" t="inlineStr">
+      <c r="GB8" s="3" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="GC8" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD8" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH8" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ8" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK8" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL8" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC8" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -5924,40 +6653,40 @@
         </is>
       </c>
       <c r="R9" s="5" t="n">
-        <v>78.8</v>
+        <v>86.8</v>
       </c>
       <c r="S9" s="5" t="n">
-        <v>68.90000000000001</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="T9" s="5" t="n">
-        <v>68.90000000000001</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="U9" s="5" t="n">
-        <v>66.5</v>
+        <v>73.5</v>
       </c>
       <c r="V9" s="5" t="n">
-        <v>66.5</v>
-      </c>
-      <c r="W9" s="6" t="n">
-        <v>56.7</v>
-      </c>
-      <c r="X9" s="7" t="n">
-        <v>56.7</v>
-      </c>
-      <c r="Y9" s="7" t="n">
-        <v>53.7</v>
+        <v>72.5</v>
+      </c>
+      <c r="W9" s="5" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="X9" s="5" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="Y9" s="6" t="n">
+        <v>57.7</v>
       </c>
       <c r="Z9" s="7" t="n">
-        <v>53.7</v>
+        <v>57.2</v>
       </c>
       <c r="AA9" s="7" t="n">
-        <v>47.3</v>
+        <v>50.3</v>
       </c>
       <c r="AB9" s="7" t="n">
-        <v>47.3</v>
+        <v>49.8</v>
       </c>
       <c r="AC9" s="7" t="n">
-        <v>42.9</v>
+        <v>43.9</v>
       </c>
       <c r="AD9" s="7" t="n">
         <v>42.9</v>
@@ -6005,7 +6734,7 @@
         <v>23.9</v>
       </c>
       <c r="AS9" s="3" t="n">
-        <v>260.64</v>
+        <v>261.36</v>
       </c>
       <c r="AT9" s="4" t="inlineStr">
         <is>
@@ -6451,7 +7180,88 @@
       <c r="GA9" s="3" t="n">
         <v>23.9</v>
       </c>
-      <c r="GB9" s="4" t="inlineStr">
+      <c r="GB9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD9" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE9" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF9" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG9" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH9" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI9" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ9" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL9" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC9" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -6530,40 +7340,40 @@
         </is>
       </c>
       <c r="R10" s="5" t="n">
-        <v>84.40000000000001</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="S10" s="5" t="n">
-        <v>79.3</v>
+        <v>87.3</v>
       </c>
       <c r="T10" s="5" t="n">
-        <v>79.3</v>
+        <v>86.8</v>
       </c>
       <c r="U10" s="5" t="n">
-        <v>74.2</v>
+        <v>81.2</v>
       </c>
       <c r="V10" s="5" t="n">
-        <v>74.2</v>
+        <v>80.2</v>
       </c>
       <c r="W10" s="5" t="n">
-        <v>66.09999999999999</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="X10" s="5" t="n">
-        <v>66.09999999999999</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="Y10" s="5" t="n">
-        <v>62.5</v>
+        <v>66.5</v>
       </c>
       <c r="Z10" s="5" t="n">
-        <v>62.5</v>
-      </c>
-      <c r="AA10" s="6" t="n">
-        <v>55.2</v>
-      </c>
-      <c r="AB10" s="7" t="n">
-        <v>55.2</v>
+        <v>66</v>
+      </c>
+      <c r="AA10" s="5" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="AB10" s="6" t="n">
+        <v>57.7</v>
       </c>
       <c r="AC10" s="7" t="n">
-        <v>51.1</v>
+        <v>52.1</v>
       </c>
       <c r="AD10" s="7" t="n">
         <v>51.1</v>
@@ -6611,7 +7421,7 @@
         <v>28</v>
       </c>
       <c r="AS10" s="3" t="n">
-        <v>260.46</v>
+        <v>261.18</v>
       </c>
       <c r="AT10" s="4" t="inlineStr">
         <is>
@@ -7051,7 +7861,88 @@
       <c r="GA10" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="GB10" s="4" t="inlineStr">
+      <c r="GB10" s="3" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="GC10" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD10" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE10" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG10" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH10" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI10" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ10" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL10" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC10" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -7130,40 +8021,40 @@
         </is>
       </c>
       <c r="R11" s="5" t="n">
-        <v>83.7</v>
+        <v>90.2</v>
       </c>
       <c r="S11" s="5" t="n">
-        <v>76.59999999999999</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="T11" s="5" t="n">
-        <v>76.59999999999999</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="U11" s="5" t="n">
-        <v>72.40000000000001</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="V11" s="5" t="n">
-        <v>72.40000000000001</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="W11" s="5" t="n">
-        <v>63.2</v>
+        <v>68.2</v>
       </c>
       <c r="X11" s="5" t="n">
-        <v>63.2</v>
+        <v>67.7</v>
       </c>
       <c r="Y11" s="5" t="n">
-        <v>59.8</v>
+        <v>63.8</v>
       </c>
       <c r="Z11" s="5" t="n">
-        <v>59.8</v>
+        <v>63.3</v>
       </c>
       <c r="AA11" s="6" t="n">
-        <v>51.7</v>
+        <v>54.7</v>
       </c>
       <c r="AB11" s="7" t="n">
-        <v>51.7</v>
+        <v>54.2</v>
       </c>
       <c r="AC11" s="7" t="n">
-        <v>47.4</v>
+        <v>48.4</v>
       </c>
       <c r="AD11" s="7" t="n">
         <v>47.4</v>
@@ -7211,7 +8102,7 @@
         <v>23.1</v>
       </c>
       <c r="AS11" s="3" t="n">
-        <v>249.41</v>
+        <v>250.13</v>
       </c>
       <c r="AT11" s="4" t="inlineStr">
         <is>
@@ -7651,7 +8542,88 @@
       <c r="GA11" s="3" t="n">
         <v>23.1</v>
       </c>
-      <c r="GB11" s="4" t="inlineStr">
+      <c r="GB11" s="3" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="GC11" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD11" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE11" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF11" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG11" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH11" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI11" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ11" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK11" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL11" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC11" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -7730,40 +8702,40 @@
         </is>
       </c>
       <c r="R12" s="5" t="n">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="S12" s="5" t="n">
-        <v>65.7</v>
+        <v>73.7</v>
       </c>
       <c r="T12" s="5" t="n">
-        <v>65.7</v>
+        <v>73.2</v>
       </c>
       <c r="U12" s="5" t="n">
-        <v>60.8</v>
+        <v>67.8</v>
       </c>
       <c r="V12" s="5" t="n">
-        <v>60.8</v>
+        <v>66.8</v>
       </c>
       <c r="W12" s="6" t="n">
-        <v>51.3</v>
+        <v>56.3</v>
       </c>
       <c r="X12" s="7" t="n">
-        <v>51.3</v>
+        <v>55.8</v>
       </c>
       <c r="Y12" s="7" t="n">
-        <v>47.9</v>
+        <v>51.9</v>
       </c>
       <c r="Z12" s="7" t="n">
-        <v>47.9</v>
+        <v>51.4</v>
       </c>
       <c r="AA12" s="7" t="n">
-        <v>41.1</v>
+        <v>44.1</v>
       </c>
       <c r="AB12" s="7" t="n">
-        <v>41.1</v>
+        <v>43.6</v>
       </c>
       <c r="AC12" s="8" t="n">
-        <v>37.4</v>
+        <v>38.4</v>
       </c>
       <c r="AD12" s="8" t="n">
         <v>37.4</v>
@@ -7811,7 +8783,7 @@
         <v>21.3</v>
       </c>
       <c r="AS12" s="3" t="n">
-        <v>247.32</v>
+        <v>248.04</v>
       </c>
       <c r="AT12" s="4" t="inlineStr">
         <is>
@@ -8257,7 +9229,88 @@
       <c r="GA12" s="3" t="n">
         <v>21.3</v>
       </c>
-      <c r="GB12" s="4" t="inlineStr">
+      <c r="GB12" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC12" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD12" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE12" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF12" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG12" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH12" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI12" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ12" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK12" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL12" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC12" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -8336,40 +9389,40 @@
         </is>
       </c>
       <c r="R13" s="5" t="n">
+        <v>87.7</v>
+      </c>
+      <c r="S13" s="5" t="n">
+        <v>80.2</v>
+      </c>
+      <c r="T13" s="5" t="n">
         <v>79.7</v>
       </c>
-      <c r="S13" s="5" t="n">
-        <v>72.2</v>
-      </c>
-      <c r="T13" s="5" t="n">
-        <v>72.2</v>
-      </c>
       <c r="U13" s="5" t="n">
-        <v>67.3</v>
+        <v>74.3</v>
       </c>
       <c r="V13" s="5" t="n">
-        <v>67.3</v>
+        <v>73.3</v>
       </c>
       <c r="W13" s="5" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="X13" s="5" t="n">
-        <v>58</v>
-      </c>
-      <c r="Y13" s="6" t="n">
-        <v>55</v>
-      </c>
-      <c r="Z13" s="7" t="n">
-        <v>55</v>
-      </c>
-      <c r="AA13" s="7" t="n">
-        <v>47.5</v>
+        <v>62.5</v>
+      </c>
+      <c r="Y13" s="5" t="n">
+        <v>59</v>
+      </c>
+      <c r="Z13" s="5" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="AA13" s="6" t="n">
+        <v>50.5</v>
       </c>
       <c r="AB13" s="7" t="n">
-        <v>47.5</v>
+        <v>50</v>
       </c>
       <c r="AC13" s="7" t="n">
-        <v>43.7</v>
+        <v>44.7</v>
       </c>
       <c r="AD13" s="7" t="n">
         <v>43.7</v>
@@ -8417,7 +9470,7 @@
         <v>22.9</v>
       </c>
       <c r="AS13" s="3" t="n">
-        <v>246.44</v>
+        <v>247.16</v>
       </c>
       <c r="AT13" s="4" t="inlineStr">
         <is>
@@ -8863,9 +9916,90 @@
       <c r="GA13" s="3" t="n">
         <v>22.9</v>
       </c>
-      <c r="GB13" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="GB13" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC13" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD13" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE13" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF13" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG13" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH13" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI13" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ13" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK13" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL13" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC13" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -8942,40 +10076,40 @@
         </is>
       </c>
       <c r="R14" s="5" t="n">
-        <v>76.8</v>
+        <v>84.8</v>
       </c>
       <c r="S14" s="5" t="n">
-        <v>67.40000000000001</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="T14" s="5" t="n">
-        <v>67.40000000000001</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="U14" s="5" t="n">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="V14" s="5" t="n">
-        <v>63</v>
-      </c>
-      <c r="W14" s="6" t="n">
-        <v>53.3</v>
-      </c>
-      <c r="X14" s="7" t="n">
-        <v>53.3</v>
+        <v>69</v>
+      </c>
+      <c r="W14" s="5" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="X14" s="6" t="n">
+        <v>57.8</v>
       </c>
       <c r="Y14" s="7" t="n">
-        <v>49.4</v>
+        <v>53.4</v>
       </c>
       <c r="Z14" s="7" t="n">
-        <v>49.4</v>
+        <v>52.9</v>
       </c>
       <c r="AA14" s="7" t="n">
-        <v>42.6</v>
+        <v>45.6</v>
       </c>
       <c r="AB14" s="7" t="n">
-        <v>42.6</v>
+        <v>45.1</v>
       </c>
       <c r="AC14" s="8" t="n">
-        <v>38.7</v>
+        <v>39.7</v>
       </c>
       <c r="AD14" s="8" t="n">
         <v>38.7</v>
@@ -9023,7 +10157,7 @@
         <v>21.8</v>
       </c>
       <c r="AS14" s="3" t="n">
-        <v>246.38</v>
+        <v>247.1</v>
       </c>
       <c r="AT14" s="4" t="inlineStr">
         <is>
@@ -9463,7 +10597,88 @@
       <c r="GA14" s="3" t="n">
         <v>21.8</v>
       </c>
-      <c r="GB14" s="4" t="inlineStr">
+      <c r="GB14" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC14" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD14" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE14" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF14" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG14" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH14" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI14" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ14" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK14" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL14" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC14" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -9542,40 +10757,40 @@
         </is>
       </c>
       <c r="R15" s="5" t="n">
-        <v>83.59999999999999</v>
+        <v>90.2</v>
       </c>
       <c r="S15" s="5" t="n">
-        <v>76.90000000000001</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="T15" s="5" t="n">
-        <v>76.90000000000001</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="U15" s="5" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="V15" s="5" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="W15" s="5" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="X15" s="5" t="n">
+        <v>67.40000000000001</v>
+      </c>
+      <c r="Y15" s="5" t="n">
         <v>62.9</v>
       </c>
-      <c r="X15" s="5" t="n">
-        <v>62.9</v>
-      </c>
-      <c r="Y15" s="5" t="n">
-        <v>58.9</v>
-      </c>
       <c r="Z15" s="5" t="n">
-        <v>58.9</v>
+        <v>62.4</v>
       </c>
       <c r="AA15" s="6" t="n">
-        <v>50.5</v>
+        <v>53.5</v>
       </c>
       <c r="AB15" s="7" t="n">
-        <v>50.5</v>
+        <v>53</v>
       </c>
       <c r="AC15" s="7" t="n">
-        <v>45.9</v>
+        <v>46.9</v>
       </c>
       <c r="AD15" s="7" t="n">
         <v>45.9</v>
@@ -9623,7 +10838,7 @@
         <v>19.2</v>
       </c>
       <c r="AS15" s="3" t="n">
-        <v>243.08</v>
+        <v>243.8</v>
       </c>
       <c r="AT15" s="4" t="inlineStr">
         <is>
@@ -10063,7 +11278,88 @@
       <c r="GA15" s="3" t="n">
         <v>19.2</v>
       </c>
-      <c r="GB15" s="4" t="inlineStr">
+      <c r="GB15" s="3" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="GC15" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD15" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE15" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF15" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG15" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH15" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI15" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ15" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK15" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL15" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC15" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -10142,40 +11438,40 @@
         </is>
       </c>
       <c r="R16" s="5" t="n">
-        <v>77.8</v>
+        <v>85.8</v>
       </c>
       <c r="S16" s="5" t="n">
-        <v>70.09999999999999</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="T16" s="5" t="n">
-        <v>70.09999999999999</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="U16" s="5" t="n">
-        <v>65.59999999999999</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="V16" s="5" t="n">
-        <v>65.59999999999999</v>
-      </c>
-      <c r="W16" s="6" t="n">
-        <v>56.1</v>
-      </c>
-      <c r="X16" s="7" t="n">
-        <v>56.1</v>
-      </c>
-      <c r="Y16" s="7" t="n">
-        <v>52.2</v>
+        <v>71.59999999999999</v>
+      </c>
+      <c r="W16" s="5" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="X16" s="5" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="Y16" s="6" t="n">
+        <v>56.2</v>
       </c>
       <c r="Z16" s="7" t="n">
-        <v>52.2</v>
+        <v>55.7</v>
       </c>
       <c r="AA16" s="7" t="n">
-        <v>44.7</v>
+        <v>47.7</v>
       </c>
       <c r="AB16" s="7" t="n">
-        <v>44.7</v>
+        <v>47.2</v>
       </c>
       <c r="AC16" s="7" t="n">
-        <v>40.3</v>
+        <v>41.3</v>
       </c>
       <c r="AD16" s="7" t="n">
         <v>40.3</v>
@@ -10223,7 +11519,7 @@
         <v>20.5</v>
       </c>
       <c r="AS16" s="3" t="n">
-        <v>237.91</v>
+        <v>238.63</v>
       </c>
       <c r="AT16" s="4" t="inlineStr">
         <is>
@@ -10669,7 +11965,88 @@
       <c r="GA16" s="3" t="n">
         <v>20.5</v>
       </c>
-      <c r="GB16" s="4" t="inlineStr">
+      <c r="GB16" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC16" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD16" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE16" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF16" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG16" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH16" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI16" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ16" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL16" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC16" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -10748,40 +12125,40 @@
         </is>
       </c>
       <c r="R17" s="5" t="n">
-        <v>84.40000000000001</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="S17" s="5" t="n">
-        <v>74.40000000000001</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="T17" s="5" t="n">
-        <v>74.40000000000001</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="U17" s="5" t="n">
-        <v>71.5</v>
+        <v>78.5</v>
       </c>
       <c r="V17" s="5" t="n">
-        <v>71.5</v>
+        <v>77.5</v>
       </c>
       <c r="W17" s="5" t="n">
-        <v>60.5</v>
+        <v>65.5</v>
       </c>
       <c r="X17" s="5" t="n">
-        <v>60.5</v>
-      </c>
-      <c r="Y17" s="6" t="n">
-        <v>56.7</v>
-      </c>
-      <c r="Z17" s="7" t="n">
-        <v>56.7</v>
-      </c>
-      <c r="AA17" s="7" t="n">
-        <v>49</v>
+        <v>65</v>
+      </c>
+      <c r="Y17" s="5" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="Z17" s="5" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="AA17" s="6" t="n">
+        <v>52</v>
       </c>
       <c r="AB17" s="7" t="n">
-        <v>49</v>
+        <v>51.5</v>
       </c>
       <c r="AC17" s="7" t="n">
-        <v>42.3</v>
+        <v>43.3</v>
       </c>
       <c r="AD17" s="7" t="n">
         <v>42.3</v>
@@ -10829,7 +12206,7 @@
         <v>14.8</v>
       </c>
       <c r="AS17" s="3" t="n">
-        <v>236.72</v>
+        <v>237.44</v>
       </c>
       <c r="AT17" s="4" t="inlineStr">
         <is>
@@ -11275,9 +12652,90 @@
       <c r="GA17" s="3" t="n">
         <v>14.8</v>
       </c>
-      <c r="GB17" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="GB17" s="3" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="GC17" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD17" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE17" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF17" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG17" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH17" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI17" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ17" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK17" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL17" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC17" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -11354,40 +12812,40 @@
         </is>
       </c>
       <c r="R18" s="5" t="n">
-        <v>72.7</v>
+        <v>80.7</v>
       </c>
       <c r="S18" s="5" t="n">
-        <v>63.2</v>
+        <v>71.2</v>
       </c>
       <c r="T18" s="5" t="n">
-        <v>63.2</v>
+        <v>70.7</v>
       </c>
       <c r="U18" s="5" t="n">
-        <v>58.5</v>
+        <v>65.5</v>
       </c>
       <c r="V18" s="5" t="n">
-        <v>58.5</v>
+        <v>64.5</v>
       </c>
       <c r="W18" s="6" t="n">
+        <v>53.9</v>
+      </c>
+      <c r="X18" s="7" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="Y18" s="7" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="Z18" s="7" t="n">
         <v>48.9</v>
       </c>
-      <c r="X18" s="7" t="n">
-        <v>48.9</v>
-      </c>
-      <c r="Y18" s="7" t="n">
-        <v>45.4</v>
-      </c>
-      <c r="Z18" s="7" t="n">
-        <v>45.4</v>
-      </c>
-      <c r="AA18" s="8" t="n">
-        <v>39.3</v>
-      </c>
-      <c r="AB18" s="8" t="n">
-        <v>39.3</v>
+      <c r="AA18" s="7" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="AB18" s="7" t="n">
+        <v>41.8</v>
       </c>
       <c r="AC18" s="8" t="n">
-        <v>35.5</v>
+        <v>36.5</v>
       </c>
       <c r="AD18" s="8" t="n">
         <v>35.5</v>
@@ -11435,7 +12893,7 @@
         <v>19.5</v>
       </c>
       <c r="AS18" s="3" t="n">
-        <v>236.66</v>
+        <v>237.38</v>
       </c>
       <c r="AT18" s="4" t="inlineStr">
         <is>
@@ -11881,7 +13339,88 @@
       <c r="GA18" s="3" t="n">
         <v>19.5</v>
       </c>
-      <c r="GB18" s="4" t="inlineStr">
+      <c r="GB18" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC18" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD18" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE18" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF18" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG18" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH18" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI18" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ18" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK18" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL18" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC18" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -11960,40 +13499,40 @@
         </is>
       </c>
       <c r="R19" s="5" t="n">
-        <v>81.90000000000001</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="S19" s="5" t="n">
-        <v>72.59999999999999</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="T19" s="5" t="n">
-        <v>72.59999999999999</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="U19" s="5" t="n">
-        <v>70.2</v>
+        <v>77.2</v>
       </c>
       <c r="V19" s="5" t="n">
-        <v>70.2</v>
+        <v>76.2</v>
       </c>
       <c r="W19" s="5" t="n">
-        <v>59.5</v>
+        <v>64.5</v>
       </c>
       <c r="X19" s="5" t="n">
-        <v>59.5</v>
-      </c>
-      <c r="Y19" s="6" t="n">
-        <v>56.1</v>
-      </c>
-      <c r="Z19" s="7" t="n">
-        <v>56.1</v>
-      </c>
-      <c r="AA19" s="7" t="n">
-        <v>49.7</v>
+        <v>64</v>
+      </c>
+      <c r="Y19" s="5" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="Z19" s="5" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="AA19" s="6" t="n">
+        <v>52.7</v>
       </c>
       <c r="AB19" s="7" t="n">
-        <v>49.7</v>
+        <v>52.2</v>
       </c>
       <c r="AC19" s="7" t="n">
-        <v>44.1</v>
+        <v>45.1</v>
       </c>
       <c r="AD19" s="7" t="n">
         <v>44.1</v>
@@ -12041,7 +13580,7 @@
         <v>21.9</v>
       </c>
       <c r="AS19" s="3" t="n">
-        <v>236.28</v>
+        <v>237</v>
       </c>
       <c r="AT19" s="4" t="inlineStr">
         <is>
@@ -12487,9 +14026,90 @@
       <c r="GA19" s="3" t="n">
         <v>21.9</v>
       </c>
-      <c r="GB19" s="4" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="GB19" s="3" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="GC19" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD19" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE19" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF19" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG19" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH19" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI19" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ19" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK19" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL19" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC19" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -12566,40 +14186,40 @@
         </is>
       </c>
       <c r="R20" s="5" t="n">
-        <v>75.90000000000001</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="S20" s="5" t="n">
-        <v>66.3</v>
+        <v>74.3</v>
       </c>
       <c r="T20" s="5" t="n">
-        <v>66.3</v>
+        <v>73.8</v>
       </c>
       <c r="U20" s="5" t="n">
-        <v>62.7</v>
+        <v>69.7</v>
       </c>
       <c r="V20" s="5" t="n">
-        <v>62.7</v>
+        <v>68.7</v>
       </c>
       <c r="W20" s="6" t="n">
-        <v>52.5</v>
+        <v>57.5</v>
       </c>
       <c r="X20" s="7" t="n">
-        <v>52.5</v>
+        <v>57</v>
       </c>
       <c r="Y20" s="7" t="n">
-        <v>49.4</v>
+        <v>53.4</v>
       </c>
       <c r="Z20" s="7" t="n">
-        <v>49.4</v>
+        <v>52.9</v>
       </c>
       <c r="AA20" s="7" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="AB20" s="7" t="n">
-        <v>43</v>
+        <v>45.5</v>
       </c>
       <c r="AC20" s="8" t="n">
-        <v>38.5</v>
+        <v>39.5</v>
       </c>
       <c r="AD20" s="8" t="n">
         <v>38.5</v>
@@ -12647,7 +14267,7 @@
         <v>18.6</v>
       </c>
       <c r="AS20" s="3" t="n">
-        <v>235.09</v>
+        <v>235.81</v>
       </c>
       <c r="AT20" s="4" t="inlineStr">
         <is>
@@ -13093,7 +14713,88 @@
       <c r="GA20" s="3" t="n">
         <v>18.6</v>
       </c>
-      <c r="GB20" s="4" t="inlineStr">
+      <c r="GB20" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC20" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD20" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE20" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF20" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG20" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH20" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI20" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ20" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK20" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL20" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC20" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -13172,40 +14873,40 @@
         </is>
       </c>
       <c r="R21" s="5" t="n">
-        <v>78.40000000000001</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="S21" s="5" t="n">
-        <v>72.09999999999999</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="T21" s="5" t="n">
-        <v>72.09999999999999</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="U21" s="5" t="n">
-        <v>65.5</v>
+        <v>72.5</v>
       </c>
       <c r="V21" s="5" t="n">
-        <v>65.5</v>
-      </c>
-      <c r="W21" s="6" t="n">
-        <v>56.8</v>
-      </c>
-      <c r="X21" s="7" t="n">
-        <v>56.8</v>
-      </c>
-      <c r="Y21" s="7" t="n">
-        <v>52.5</v>
+        <v>71.5</v>
+      </c>
+      <c r="W21" s="5" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="X21" s="5" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="Y21" s="6" t="n">
+        <v>56.5</v>
       </c>
       <c r="Z21" s="7" t="n">
-        <v>52.5</v>
+        <v>56</v>
       </c>
       <c r="AA21" s="7" t="n">
-        <v>44.5</v>
+        <v>47.5</v>
       </c>
       <c r="AB21" s="7" t="n">
-        <v>44.5</v>
+        <v>47</v>
       </c>
       <c r="AC21" s="7" t="n">
-        <v>41.1</v>
+        <v>42.1</v>
       </c>
       <c r="AD21" s="7" t="n">
         <v>41.1</v>
@@ -13253,7 +14954,7 @@
         <v>19.8</v>
       </c>
       <c r="AS21" s="3" t="n">
-        <v>234.12</v>
+        <v>234.84</v>
       </c>
       <c r="AT21" s="4" t="inlineStr">
         <is>
@@ -13699,7 +15400,88 @@
       <c r="GA21" s="3" t="n">
         <v>19.8</v>
       </c>
-      <c r="GB21" s="4" t="inlineStr">
+      <c r="GB21" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC21" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD21" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE21" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF21" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG21" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH21" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI21" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ21" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK21" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL21" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC21" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -13778,40 +15560,40 @@
         </is>
       </c>
       <c r="R22" s="5" t="n">
-        <v>73.90000000000001</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="S22" s="5" t="n">
-        <v>65.3</v>
+        <v>73.3</v>
       </c>
       <c r="T22" s="5" t="n">
-        <v>65.3</v>
+        <v>72.8</v>
       </c>
       <c r="U22" s="5" t="n">
-        <v>60.4</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="V22" s="5" t="n">
-        <v>60.4</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="W22" s="6" t="n">
-        <v>50.2</v>
+        <v>55.2</v>
       </c>
       <c r="X22" s="7" t="n">
-        <v>50.2</v>
+        <v>54.7</v>
       </c>
       <c r="Y22" s="7" t="n">
-        <v>47.3</v>
+        <v>51.3</v>
       </c>
       <c r="Z22" s="7" t="n">
-        <v>47.3</v>
-      </c>
-      <c r="AA22" s="8" t="n">
-        <v>39.6</v>
-      </c>
-      <c r="AB22" s="8" t="n">
-        <v>39.6</v>
+        <v>50.8</v>
+      </c>
+      <c r="AA22" s="7" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="AB22" s="7" t="n">
+        <v>42.1</v>
       </c>
       <c r="AC22" s="8" t="n">
-        <v>35.9</v>
+        <v>36.9</v>
       </c>
       <c r="AD22" s="8" t="n">
         <v>35.9</v>
@@ -13859,7 +15641,7 @@
         <v>18</v>
       </c>
       <c r="AS22" s="3" t="n">
-        <v>233.48</v>
+        <v>234.2</v>
       </c>
       <c r="AT22" s="4" t="inlineStr">
         <is>
@@ -14305,7 +16087,88 @@
       <c r="GA22" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="GB22" s="4" t="inlineStr">
+      <c r="GB22" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC22" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD22" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE22" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF22" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG22" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH22" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI22" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ22" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK22" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL22" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC22" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -14384,40 +16247,40 @@
         </is>
       </c>
       <c r="R23" s="5" t="n">
-        <v>73.90000000000001</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="S23" s="5" t="n">
-        <v>67.8</v>
+        <v>75.8</v>
       </c>
       <c r="T23" s="5" t="n">
-        <v>67.8</v>
+        <v>75.3</v>
       </c>
       <c r="U23" s="5" t="n">
-        <v>60.9</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="V23" s="5" t="n">
-        <v>60.9</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="W23" s="6" t="n">
-        <v>52.8</v>
+        <v>57.8</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>52.8</v>
+        <v>57.3</v>
       </c>
       <c r="Y23" s="7" t="n">
-        <v>48.5</v>
+        <v>52.5</v>
       </c>
       <c r="Z23" s="7" t="n">
-        <v>48.5</v>
+        <v>52</v>
       </c>
       <c r="AA23" s="7" t="n">
-        <v>41.6</v>
+        <v>44.6</v>
       </c>
       <c r="AB23" s="7" t="n">
-        <v>41.6</v>
+        <v>44.1</v>
       </c>
       <c r="AC23" s="8" t="n">
-        <v>38.2</v>
+        <v>39.2</v>
       </c>
       <c r="AD23" s="8" t="n">
         <v>38.2</v>
@@ -14465,7 +16328,7 @@
         <v>20.8</v>
       </c>
       <c r="AS23" s="3" t="n">
-        <v>231.86</v>
+        <v>232.58</v>
       </c>
       <c r="AT23" s="4" t="inlineStr">
         <is>
@@ -14905,7 +16768,88 @@
       <c r="GA23" s="3" t="n">
         <v>20.8</v>
       </c>
-      <c r="GB23" s="4" t="inlineStr">
+      <c r="GB23" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC23" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD23" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE23" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF23" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG23" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH23" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI23" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ23" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK23" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL23" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC23" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -14984,40 +16928,40 @@
         </is>
       </c>
       <c r="R24" s="5" t="n">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="S24" s="5" t="n">
-        <v>71.7</v>
+        <v>79.7</v>
       </c>
       <c r="T24" s="5" t="n">
-        <v>71.7</v>
+        <v>79.2</v>
       </c>
       <c r="U24" s="5" t="n">
-        <v>66.7</v>
+        <v>73.7</v>
       </c>
       <c r="V24" s="5" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="W24" s="6" t="n">
-        <v>57</v>
-      </c>
-      <c r="X24" s="7" t="n">
-        <v>57</v>
-      </c>
-      <c r="Y24" s="7" t="n">
-        <v>53.6</v>
+        <v>72.7</v>
+      </c>
+      <c r="W24" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="X24" s="5" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="Y24" s="6" t="n">
+        <v>57.6</v>
       </c>
       <c r="Z24" s="7" t="n">
-        <v>53.6</v>
+        <v>57.1</v>
       </c>
       <c r="AA24" s="7" t="n">
-        <v>45.8</v>
+        <v>48.8</v>
       </c>
       <c r="AB24" s="7" t="n">
-        <v>45.8</v>
+        <v>48.3</v>
       </c>
       <c r="AC24" s="7" t="n">
-        <v>41.8</v>
+        <v>42.8</v>
       </c>
       <c r="AD24" s="7" t="n">
         <v>41.8</v>
@@ -15065,7 +17009,7 @@
         <v>21.7</v>
       </c>
       <c r="AS24" s="3" t="n">
-        <v>230.73</v>
+        <v>231.45</v>
       </c>
       <c r="AT24" s="4" t="inlineStr">
         <is>
@@ -15505,7 +17449,88 @@
       <c r="GA24" s="3" t="n">
         <v>21.7</v>
       </c>
-      <c r="GB24" s="4" t="inlineStr">
+      <c r="GB24" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC24" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD24" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE24" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF24" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG24" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH24" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI24" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ24" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK24" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL24" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC24" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -15584,40 +17609,40 @@
         </is>
       </c>
       <c r="R25" s="5" t="n">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="S25" s="5" t="n">
-        <v>66.40000000000001</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="T25" s="5" t="n">
-        <v>66.40000000000001</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="U25" s="5" t="n">
-        <v>60.5</v>
+        <v>67.5</v>
       </c>
       <c r="V25" s="5" t="n">
-        <v>60.5</v>
+        <v>66.5</v>
       </c>
       <c r="W25" s="6" t="n">
-        <v>51.7</v>
+        <v>56.7</v>
       </c>
       <c r="X25" s="7" t="n">
-        <v>51.7</v>
+        <v>56.2</v>
       </c>
       <c r="Y25" s="7" t="n">
-        <v>48.5</v>
+        <v>52.5</v>
       </c>
       <c r="Z25" s="7" t="n">
-        <v>48.5</v>
+        <v>52</v>
       </c>
       <c r="AA25" s="7" t="n">
-        <v>41.3</v>
+        <v>44.3</v>
       </c>
       <c r="AB25" s="7" t="n">
-        <v>41.3</v>
+        <v>43.8</v>
       </c>
       <c r="AC25" s="8" t="n">
-        <v>37.8</v>
+        <v>38.8</v>
       </c>
       <c r="AD25" s="8" t="n">
         <v>37.8</v>
@@ -15665,7 +17690,7 @@
         <v>19.2</v>
       </c>
       <c r="AS25" s="3" t="n">
-        <v>227.05</v>
+        <v>227.77</v>
       </c>
       <c r="AT25" s="4" t="inlineStr">
         <is>
@@ -16105,7 +18130,88 @@
       <c r="GA25" s="3" t="n">
         <v>19.2</v>
       </c>
-      <c r="GB25" s="4" t="inlineStr">
+      <c r="GB25" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC25" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD25" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE25" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF25" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG25" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH25" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI25" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ25" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK25" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL25" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC25" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -16184,40 +18290,40 @@
         </is>
       </c>
       <c r="R26" s="5" t="n">
-        <v>74.5</v>
+        <v>82.5</v>
       </c>
       <c r="S26" s="5" t="n">
-        <v>65.59999999999999</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="T26" s="5" t="n">
-        <v>65.59999999999999</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="U26" s="5" t="n">
-        <v>60.3</v>
+        <v>67.3</v>
       </c>
       <c r="V26" s="5" t="n">
-        <v>60.3</v>
+        <v>66.3</v>
       </c>
       <c r="W26" s="6" t="n">
-        <v>50.7</v>
+        <v>55.7</v>
       </c>
       <c r="X26" s="7" t="n">
-        <v>50.7</v>
+        <v>55.2</v>
       </c>
       <c r="Y26" s="7" t="n">
-        <v>47.1</v>
+        <v>51.1</v>
       </c>
       <c r="Z26" s="7" t="n">
-        <v>47.1</v>
+        <v>50.6</v>
       </c>
       <c r="AA26" s="7" t="n">
-        <v>40.6</v>
+        <v>43.6</v>
       </c>
       <c r="AB26" s="7" t="n">
-        <v>40.6</v>
+        <v>43.1</v>
       </c>
       <c r="AC26" s="8" t="n">
-        <v>36.7</v>
+        <v>37.7</v>
       </c>
       <c r="AD26" s="8" t="n">
         <v>36.7</v>
@@ -16265,7 +18371,7 @@
         <v>20.4</v>
       </c>
       <c r="AS26" s="3" t="n">
-        <v>226.93</v>
+        <v>227.65</v>
       </c>
       <c r="AT26" s="4" t="inlineStr">
         <is>
@@ -16711,7 +18817,88 @@
       <c r="GA26" s="3" t="n">
         <v>20.4</v>
       </c>
-      <c r="GB26" s="4" t="inlineStr">
+      <c r="GB26" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC26" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD26" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE26" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF26" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG26" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH26" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI26" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ26" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK26" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL26" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC26" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -16790,40 +18977,40 @@
         </is>
       </c>
       <c r="R27" s="5" t="n">
-        <v>75.5</v>
+        <v>83.5</v>
       </c>
       <c r="S27" s="5" t="n">
-        <v>68.3</v>
+        <v>76.3</v>
       </c>
       <c r="T27" s="5" t="n">
-        <v>68.3</v>
+        <v>75.8</v>
       </c>
       <c r="U27" s="5" t="n">
-        <v>62.8</v>
+        <v>69.8</v>
       </c>
       <c r="V27" s="5" t="n">
-        <v>62.8</v>
-      </c>
-      <c r="W27" s="6" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="W27" s="5" t="n">
+        <v>59</v>
+      </c>
+      <c r="X27" s="5" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="Y27" s="6" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="Z27" s="7" t="n">
         <v>54</v>
       </c>
-      <c r="X27" s="7" t="n">
-        <v>54</v>
-      </c>
-      <c r="Y27" s="7" t="n">
-        <v>50.5</v>
-      </c>
-      <c r="Z27" s="7" t="n">
-        <v>50.5</v>
-      </c>
       <c r="AA27" s="7" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="AB27" s="7" t="n">
-        <v>43</v>
-      </c>
-      <c r="AC27" s="8" t="n">
-        <v>39.5</v>
+        <v>45.5</v>
+      </c>
+      <c r="AC27" s="7" t="n">
+        <v>40.5</v>
       </c>
       <c r="AD27" s="8" t="n">
         <v>39.5</v>
@@ -16871,7 +19058,7 @@
         <v>20.7</v>
       </c>
       <c r="AS27" s="3" t="n">
-        <v>223.54</v>
+        <v>224.26</v>
       </c>
       <c r="AT27" s="4" t="inlineStr">
         <is>
@@ -17311,7 +19498,88 @@
       <c r="GA27" s="3" t="n">
         <v>20.7</v>
       </c>
-      <c r="GB27" s="4" t="inlineStr">
+      <c r="GB27" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC27" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD27" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE27" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF27" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG27" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH27" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI27" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ27" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK27" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL27" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC27" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -17390,40 +19658,40 @@
         </is>
       </c>
       <c r="R28" s="5" t="n">
-        <v>75.2</v>
+        <v>83.2</v>
       </c>
       <c r="S28" s="5" t="n">
-        <v>65.8</v>
+        <v>73.8</v>
       </c>
       <c r="T28" s="5" t="n">
-        <v>65.8</v>
+        <v>73.3</v>
       </c>
       <c r="U28" s="5" t="n">
-        <v>61.1</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="V28" s="5" t="n">
-        <v>61.1</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="W28" s="6" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="X28" s="7" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Y28" s="7" t="n">
         <v>50.4</v>
       </c>
-      <c r="X28" s="7" t="n">
-        <v>50.4</v>
-      </c>
-      <c r="Y28" s="7" t="n">
-        <v>46.4</v>
-      </c>
       <c r="Z28" s="7" t="n">
-        <v>46.4</v>
-      </c>
-      <c r="AA28" s="8" t="n">
-        <v>38.4</v>
-      </c>
-      <c r="AB28" s="8" t="n">
-        <v>38.4</v>
+        <v>49.9</v>
+      </c>
+      <c r="AA28" s="7" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="AB28" s="7" t="n">
+        <v>40.9</v>
       </c>
       <c r="AC28" s="8" t="n">
-        <v>33.4</v>
+        <v>34.4</v>
       </c>
       <c r="AD28" s="8" t="n">
         <v>33.4</v>
@@ -17471,7 +19739,7 @@
         <v>12.8</v>
       </c>
       <c r="AS28" s="3" t="n">
-        <v>222.21</v>
+        <v>222.93</v>
       </c>
       <c r="AT28" s="4" t="inlineStr">
         <is>
@@ -17911,7 +20179,88 @@
       <c r="GA28" s="3" t="n">
         <v>12.8</v>
       </c>
-      <c r="GB28" s="4" t="inlineStr">
+      <c r="GB28" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC28" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD28" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE28" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF28" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG28" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH28" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI28" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ28" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK28" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL28" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC28" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -17990,40 +20339,40 @@
         </is>
       </c>
       <c r="R29" s="5" t="n">
-        <v>71.90000000000001</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="S29" s="5" t="n">
-        <v>64.3</v>
+        <v>72.3</v>
       </c>
       <c r="T29" s="5" t="n">
-        <v>64.3</v>
-      </c>
-      <c r="U29" s="6" t="n">
-        <v>57.7</v>
-      </c>
-      <c r="V29" s="7" t="n">
-        <v>57.7</v>
-      </c>
-      <c r="W29" s="7" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="U29" s="5" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="V29" s="5" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="W29" s="6" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="X29" s="7" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="Y29" s="7" t="n">
         <v>48.8</v>
       </c>
-      <c r="X29" s="7" t="n">
-        <v>48.8</v>
-      </c>
-      <c r="Y29" s="7" t="n">
-        <v>44.8</v>
-      </c>
       <c r="Z29" s="7" t="n">
-        <v>44.8</v>
-      </c>
-      <c r="AA29" s="8" t="n">
-        <v>37.9</v>
-      </c>
-      <c r="AB29" s="8" t="n">
-        <v>37.9</v>
+        <v>48.3</v>
+      </c>
+      <c r="AA29" s="7" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="AB29" s="7" t="n">
+        <v>40.4</v>
       </c>
       <c r="AC29" s="8" t="n">
-        <v>34.6</v>
+        <v>35.6</v>
       </c>
       <c r="AD29" s="8" t="n">
         <v>34.6</v>
@@ -18071,7 +20420,7 @@
         <v>17.8</v>
       </c>
       <c r="AS29" s="3" t="n">
-        <v>221.49</v>
+        <v>222.21</v>
       </c>
       <c r="AT29" s="4" t="inlineStr">
         <is>
@@ -18517,7 +20866,88 @@
       <c r="GA29" s="3" t="n">
         <v>17.8</v>
       </c>
-      <c r="GB29" s="4" t="inlineStr">
+      <c r="GB29" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC29" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD29" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE29" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF29" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG29" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH29" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI29" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ29" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK29" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL29" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC29" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -18596,40 +21026,40 @@
         </is>
       </c>
       <c r="R30" s="5" t="n">
-        <v>72.3</v>
+        <v>80.3</v>
       </c>
       <c r="S30" s="5" t="n">
-        <v>62.3</v>
+        <v>70.3</v>
       </c>
       <c r="T30" s="5" t="n">
-        <v>62.3</v>
+        <v>69.8</v>
       </c>
       <c r="U30" s="5" t="n">
-        <v>58.7</v>
+        <v>65.7</v>
       </c>
       <c r="V30" s="5" t="n">
-        <v>58.7</v>
+        <v>64.7</v>
       </c>
       <c r="W30" s="6" t="n">
-        <v>48.1</v>
+        <v>53.1</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>48.1</v>
+        <v>52.6</v>
       </c>
       <c r="Y30" s="7" t="n">
-        <v>45.2</v>
+        <v>49.2</v>
       </c>
       <c r="Z30" s="7" t="n">
-        <v>45.2</v>
-      </c>
-      <c r="AA30" s="8" t="n">
-        <v>38.4</v>
-      </c>
-      <c r="AB30" s="8" t="n">
-        <v>38.4</v>
+        <v>48.7</v>
+      </c>
+      <c r="AA30" s="7" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="AB30" s="7" t="n">
+        <v>40.9</v>
       </c>
       <c r="AC30" s="8" t="n">
-        <v>34.3</v>
+        <v>35.3</v>
       </c>
       <c r="AD30" s="8" t="n">
         <v>34.3</v>
@@ -18677,7 +21107,7 @@
         <v>16.8</v>
       </c>
       <c r="AS30" s="3" t="n">
-        <v>220.75</v>
+        <v>221.47</v>
       </c>
       <c r="AT30" s="4" t="inlineStr">
         <is>
@@ -19123,7 +21553,88 @@
       <c r="GA30" s="3" t="n">
         <v>16.8</v>
       </c>
-      <c r="GB30" s="4" t="inlineStr">
+      <c r="GB30" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC30" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD30" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE30" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF30" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG30" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH30" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI30" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ30" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK30" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL30" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC30" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -19202,40 +21713,40 @@
         </is>
       </c>
       <c r="R31" s="5" t="n">
-        <v>65.09999999999999</v>
-      </c>
-      <c r="S31" s="6" t="n">
-        <v>54.1</v>
-      </c>
-      <c r="T31" s="7" t="n">
-        <v>54.1</v>
-      </c>
-      <c r="U31" s="7" t="n">
-        <v>50.9</v>
+        <v>73.09999999999999</v>
+      </c>
+      <c r="S31" s="5" t="n">
+        <v>62.1</v>
+      </c>
+      <c r="T31" s="5" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="U31" s="6" t="n">
+        <v>57.9</v>
       </c>
       <c r="V31" s="7" t="n">
-        <v>50.9</v>
+        <v>56.9</v>
       </c>
       <c r="W31" s="7" t="n">
-        <v>41.7</v>
+        <v>46.7</v>
       </c>
       <c r="X31" s="7" t="n">
-        <v>41.7</v>
-      </c>
-      <c r="Y31" s="8" t="n">
-        <v>39</v>
-      </c>
-      <c r="Z31" s="8" t="n">
-        <v>39</v>
+        <v>46.2</v>
+      </c>
+      <c r="Y31" s="7" t="n">
+        <v>43</v>
+      </c>
+      <c r="Z31" s="7" t="n">
+        <v>42.5</v>
       </c>
       <c r="AA31" s="8" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="AB31" s="8" t="n">
-        <v>34</v>
+        <v>36.5</v>
       </c>
       <c r="AC31" s="8" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="AD31" s="8" t="n">
         <v>31</v>
@@ -19283,7 +21794,7 @@
         <v>18.1</v>
       </c>
       <c r="AS31" s="3" t="n">
-        <v>219.62</v>
+        <v>220.34</v>
       </c>
       <c r="AT31" s="4" t="inlineStr">
         <is>
@@ -19723,14 +22234,95 @@
       <c r="GA31" s="3" t="n">
         <v>18.1</v>
       </c>
-      <c r="GB31" s="4" t="inlineStr">
+      <c r="GB31" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GC31" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="GD31" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="GE31" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="GF31" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="GG31" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="GH31" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="GI31" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="GJ31" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="GK31" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="GL31" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="GM31" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="GN31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GO31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GP31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GQ31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GR31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GS31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GT31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GU31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GV31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GW31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GX31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="GZ31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HA31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HB31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC31" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:GB31"/>
+  <autoFilter ref="A1:HC31"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>